<commit_message>
add observation page and initial functions and logic
</commit_message>
<xml_diff>
--- a/notebooks/Performance Report - 2023Q1 - January – March 2023.xlsx
+++ b/notebooks/Performance Report - 2023Q1 - January – March 2023.xlsx
@@ -11,8 +11,6 @@
     <sheet name="Sales Analysis" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Chart Data" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="observations" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="observations1" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="observations2" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,6 +492,125 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Chart Data'!X2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Chart Data'!$V$3:$W$93</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$X$3:$X$93</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Chart Data'!Y2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Chart Data'!$V$3:$W$93</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$Y$3:$Y$93</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Chart Data'!Z2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Chart Data'!$V$3:$W$93</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Chart Data'!$Z$3:$Z$93</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+        <noMultiLvlLbl val="0"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="tr"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -579,6 +696,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12240000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1002,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1046,6 +1185,9 @@
       </c>
     </row>
     <row r="5" ht="283.5" customHeight="1"/>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" t="inlineStr"/>
+    </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1059,34 +1201,22 @@
       </c>
     </row>
     <row r="8" ht="283.5" customHeight="1"/>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" t="inlineStr"/>
+    </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Key Observations</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Key Observations</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Key Observations</t>
-        </is>
-      </c>
-    </row>
+          <t>Comparative Location Performance Grouped by Hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="255.15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A19:I19"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A28:I28"/>
-    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1099,7 +1229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK92"/>
+  <dimension ref="A1:Z93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1163,11 +1293,6 @@
           <t>Lower Manhattan Revenue</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Lower Manhattan</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1214,82 +1339,27 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
+          <t>Hour</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>Astoria</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Hell's Kitchen</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>20:00</t>
+          <t>Lower Manhattan</t>
         </is>
       </c>
     </row>
@@ -1338,53 +1408,22 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="W3" t="n">
-        <v>222</v>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
       </c>
       <c r="X3" t="n">
-        <v>1841.13</v>
+        <v>1211.05</v>
       </c>
       <c r="Y3" t="n">
+        <v>2144.9</v>
+      </c>
+      <c r="Z3" t="n">
         <v>1728.71</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1726.18</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>1751.82</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>731.91</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>898.89</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>549.38</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>845.33</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>955.29</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>868.63</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>693.45</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>374.04</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>60.51</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -1430,55 +1469,20 @@
       <c r="T4" t="n">
         <v>1127.55</v>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="W4" t="n">
-        <v>450.2</v>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
       </c>
       <c r="X4" t="n">
-        <v>1614.94</v>
+        <v>1394.15</v>
       </c>
       <c r="Y4" t="n">
+        <v>2199.28</v>
+      </c>
+      <c r="Z4" t="n">
         <v>1488.8</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>1681.15</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>1760.25</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>627.95</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>555.55</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>687.25</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>661.05</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>518.75</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>576.15</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>398.85</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>210.95</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="5">
@@ -1516,55 +1520,20 @@
       <c r="T5" t="n">
         <v>1092</v>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="W5" t="n">
-        <v>915.55</v>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
       </c>
       <c r="X5" t="n">
-        <v>1325.66</v>
+        <v>1177.45</v>
       </c>
       <c r="Y5" t="n">
+        <v>1357.45</v>
+      </c>
+      <c r="Z5" t="n">
         <v>1443.5</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1410.7</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>1410.55</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>566.05</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>771.45</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>752.75</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>640.03</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>894</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>728.65</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>637.05</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>383.85</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>84.95</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>46.5</v>
       </c>
     </row>
     <row r="6">
@@ -1594,55 +1563,20 @@
       <c r="T6" t="n">
         <v>1202.25</v>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="W6" t="n">
-        <v>1077.65</v>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
       </c>
       <c r="X6" t="n">
-        <v>1311.44</v>
+        <v>1156.08</v>
       </c>
       <c r="Y6" t="n">
+        <v>1554.25</v>
+      </c>
+      <c r="Z6" t="n">
         <v>1379.45</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>1593.87</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>1689.77</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>666.7</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>768.48</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>535.23</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>677.25</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>734.78</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>708.05</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>693.38</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>413.75</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>116.02</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>33.77</v>
       </c>
     </row>
     <row r="7">
@@ -1672,55 +1606,20 @@
       <c r="T7" t="n">
         <v>1080.25</v>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="W7" t="n">
-        <v>826.2</v>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
       </c>
       <c r="X7" t="n">
-        <v>1747.7</v>
+        <v>1108.9</v>
       </c>
       <c r="Y7" t="n">
+        <v>1754.58</v>
+      </c>
+      <c r="Z7" t="n">
         <v>1510.83</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>1470.6</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>1632.75</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>874.5</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>736.9</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>530.85</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>841.8</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>865.05</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>776.5</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>669.2</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>273.7</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1750,55 +1649,20 @@
       <c r="T8" t="n">
         <v>1014.75</v>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="W8" t="n">
-        <v>785.75</v>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
       </c>
       <c r="X8" t="n">
-        <v>1560.63</v>
+        <v>1167.8</v>
       </c>
       <c r="Y8" t="n">
+        <v>1972.63</v>
+      </c>
+      <c r="Z8" t="n">
         <v>1386.5</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>1365.9</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>1314.65</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>568.05</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>671.3</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>737.25</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>725.1799999999999</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>691.8</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>620.65</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>448.45</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>282.8</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1828,55 +1692,20 @@
       <c r="T9" t="n">
         <v>1513.35</v>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="W9" t="n">
-        <v>971.5</v>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
       </c>
       <c r="X9" t="n">
-        <v>1396.73</v>
+        <v>1227.11</v>
       </c>
       <c r="Y9" t="n">
+        <v>1246.5</v>
+      </c>
+      <c r="Z9" t="n">
         <v>1315</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>1436.5</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>1483.45</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>744.95</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>730.5</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>737.75</v>
-      </c>
-      <c r="AE9" t="n">
-        <v>688.15</v>
-      </c>
-      <c r="AF9" t="n">
-        <v>769.05</v>
-      </c>
-      <c r="AG9" t="n">
-        <v>622.1</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>578.45</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>390.95</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>31.05</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>39.4</v>
       </c>
     </row>
     <row r="10">
@@ -1908,8 +1737,22 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Hell's Kitchen</t>
-        </is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>990.95</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>2049.85</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1726.18</v>
       </c>
     </row>
     <row r="11">
@@ -1931,85 +1774,20 @@
       <c r="T11" t="n">
         <v>1453.8</v>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="AJ11" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="AK11" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>1565.63</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>2555.7</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>1681.15</v>
       </c>
     </row>
     <row r="12">
@@ -2031,55 +1809,20 @@
       <c r="T12" t="n">
         <v>1195.83</v>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="W12" t="n">
-        <v>188.9</v>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
       </c>
       <c r="X12" t="n">
-        <v>416.25</v>
+        <v>1268.8</v>
       </c>
       <c r="Y12" t="n">
-        <v>2144.9</v>
+        <v>1333.75</v>
       </c>
       <c r="Z12" t="n">
-        <v>2049.85</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>2078.45</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>751.2</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>665.3</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>616.35</v>
-      </c>
-      <c r="AE12" t="n">
-        <v>734.3</v>
-      </c>
-      <c r="AF12" t="n">
-        <v>622.1</v>
-      </c>
-      <c r="AG12" t="n">
-        <v>675.9</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>655</v>
-      </c>
-      <c r="AI12" t="n">
-        <v>516.45</v>
-      </c>
-      <c r="AJ12" t="n">
-        <v>524.2</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>287.1</v>
+        <v>1410.7</v>
       </c>
     </row>
     <row r="13">
@@ -2101,55 +1844,20 @@
       <c r="T13" t="n">
         <v>1512.55</v>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="W13" t="n">
-        <v>202.15</v>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
       </c>
       <c r="X13" t="n">
-        <v>351.75</v>
+        <v>1210.3</v>
       </c>
       <c r="Y13" t="n">
-        <v>2199.28</v>
+        <v>1421</v>
       </c>
       <c r="Z13" t="n">
-        <v>2555.7</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>1884.55</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>680.1</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>541.65</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>693.85</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>607.2</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>598.55</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>713.55</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>753.15</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>562.25</v>
-      </c>
-      <c r="AJ13" t="n">
-        <v>552</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>339.5</v>
+        <v>1593.87</v>
       </c>
     </row>
     <row r="14">
@@ -2171,55 +1879,20 @@
       <c r="T14" t="n">
         <v>1247.43</v>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="W14" t="n">
-        <v>433.4</v>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
       </c>
       <c r="X14" t="n">
-        <v>1011.1</v>
+        <v>1199</v>
       </c>
       <c r="Y14" t="n">
-        <v>1357.45</v>
+        <v>1634.9</v>
       </c>
       <c r="Z14" t="n">
-        <v>1333.75</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>1354.15</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>1122.45</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>559.5</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>611.1</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>710.9299999999999</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>534.35</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>652.46</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>755.55</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>708.35</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>605.35</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>0</v>
+        <v>1470.6</v>
       </c>
     </row>
     <row r="15">
@@ -2241,55 +1914,20 @@
       <c r="T15" t="n">
         <v>1116.96</v>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="W15" t="n">
-        <v>642.5</v>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
       </c>
       <c r="X15" t="n">
-        <v>1277.1</v>
+        <v>1131.5</v>
       </c>
       <c r="Y15" t="n">
-        <v>1554.25</v>
+        <v>1458.45</v>
       </c>
       <c r="Z15" t="n">
-        <v>1421</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>1588.94</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>1146.66</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>469.65</v>
-      </c>
-      <c r="AD15" t="n">
-        <v>615.5</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>659.25</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>623.35</v>
-      </c>
-      <c r="AG15" t="n">
-        <v>558.8</v>
-      </c>
-      <c r="AH15" t="n">
-        <v>745.75</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>648.38</v>
-      </c>
-      <c r="AJ15" t="n">
-        <v>520.1</v>
-      </c>
-      <c r="AK15" t="n">
-        <v>11.85</v>
+        <v>1365.9</v>
       </c>
     </row>
     <row r="16">
@@ -2311,55 +1949,20 @@
       <c r="T16" t="n">
         <v>1270.05</v>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="W16" t="n">
-        <v>417.25</v>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
       </c>
       <c r="X16" t="n">
-        <v>813.25</v>
+        <v>1329.9</v>
       </c>
       <c r="Y16" t="n">
-        <v>1754.58</v>
+        <v>1578.05</v>
       </c>
       <c r="Z16" t="n">
-        <v>1634.9</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>1741.85</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>684.65</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>662.7</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>524.55</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>631.8</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>718.45</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>688.4</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>629</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>750.45</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>506.15</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>111.1</v>
+        <v>1436.5</v>
       </c>
     </row>
     <row r="17">
@@ -2383,53 +1986,22 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="W17" t="n">
-        <v>377.55</v>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
       </c>
       <c r="X17" t="n">
-        <v>777.55</v>
+        <v>1297.68</v>
       </c>
       <c r="Y17" t="n">
-        <v>1972.63</v>
+        <v>2078.45</v>
       </c>
       <c r="Z17" t="n">
-        <v>1458.45</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>1922.45</v>
-      </c>
-      <c r="AB17" t="n">
-        <v>755.13</v>
-      </c>
-      <c r="AC17" t="n">
-        <v>583.05</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>567.4</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>639.85</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>433.9</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>581.65</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>573.95</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>570.3</v>
-      </c>
-      <c r="AJ17" t="n">
-        <v>550.78</v>
-      </c>
-      <c r="AK17" t="n">
-        <v>135.88</v>
+        <v>1751.82</v>
       </c>
     </row>
     <row r="18">
@@ -2451,55 +2023,20 @@
       <c r="T18" t="n">
         <v>1150.05</v>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="W18" t="n">
-        <v>486.53</v>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
       </c>
       <c r="X18" t="n">
-        <v>1192.8</v>
+        <v>1353.35</v>
       </c>
       <c r="Y18" t="n">
-        <v>1246.5</v>
+        <v>1884.55</v>
       </c>
       <c r="Z18" t="n">
-        <v>1578.05</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>1547.9</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>837.9</v>
-      </c>
-      <c r="AC18" t="n">
-        <v>556.75</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>616.15</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>670.78</v>
-      </c>
-      <c r="AF18" t="n">
-        <v>508.4</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>735.28</v>
-      </c>
-      <c r="AH18" t="n">
-        <v>839.05</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>657.1799999999999</v>
-      </c>
-      <c r="AJ18" t="n">
-        <v>613.7</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>0</v>
+        <v>1760.25</v>
       </c>
     </row>
     <row r="19">
@@ -2521,10 +2058,20 @@
       <c r="T19" t="n">
         <v>1164.68</v>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>Astoria</t>
-        </is>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>1205.45</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>1354.15</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>1410.55</v>
       </c>
     </row>
     <row r="20">
@@ -2546,75 +2093,20 @@
       <c r="T20" t="n">
         <v>1130.2</v>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
-          <t>07:00</t>
-        </is>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="AB20" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="AE20" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="AF20" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="AG20" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="AH20" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="AI20" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X20" t="n">
+        <v>1159.2</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>1588.94</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>1689.77</v>
       </c>
     </row>
     <row r="21">
@@ -2636,49 +2128,20 @@
       <c r="T21" t="n">
         <v>1443.43</v>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="W21" t="n">
-        <v>1007.15</v>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
       </c>
       <c r="X21" t="n">
-        <v>1211.05</v>
+        <v>1437.8</v>
       </c>
       <c r="Y21" t="n">
-        <v>990.95</v>
+        <v>1741.85</v>
       </c>
       <c r="Z21" t="n">
-        <v>1297.68</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>703.63</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>811.75</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>643.03</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>849.9</v>
-      </c>
-      <c r="AE21" t="n">
-        <v>796.55</v>
-      </c>
-      <c r="AF21" t="n">
-        <v>743.9</v>
-      </c>
-      <c r="AG21" t="n">
-        <v>827.55</v>
-      </c>
-      <c r="AH21" t="n">
-        <v>714.55</v>
-      </c>
-      <c r="AI21" t="n">
-        <v>733.3099999999999</v>
+        <v>1632.75</v>
       </c>
     </row>
     <row r="22">
@@ -2700,49 +2163,20 @@
       <c r="T22" t="n">
         <v>1381.65</v>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="W22" t="n">
-        <v>920.4</v>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
       </c>
       <c r="X22" t="n">
-        <v>1394.15</v>
+        <v>1356.75</v>
       </c>
       <c r="Y22" t="n">
-        <v>1565.63</v>
+        <v>1922.45</v>
       </c>
       <c r="Z22" t="n">
-        <v>1353.35</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>779.75</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>564.95</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>712.6</v>
-      </c>
-      <c r="AD22" t="n">
-        <v>609.65</v>
-      </c>
-      <c r="AE22" t="n">
-        <v>727.75</v>
-      </c>
-      <c r="AF22" t="n">
-        <v>662.5</v>
-      </c>
-      <c r="AG22" t="n">
-        <v>753.55</v>
-      </c>
-      <c r="AH22" t="n">
-        <v>735.9</v>
-      </c>
-      <c r="AI22" t="n">
-        <v>811.7</v>
+        <v>1314.65</v>
       </c>
     </row>
     <row r="23">
@@ -2764,49 +2198,20 @@
       <c r="T23" t="n">
         <v>1634.18</v>
       </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="W23" t="n">
-        <v>1122.18</v>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
       </c>
       <c r="X23" t="n">
-        <v>1177.45</v>
+        <v>1364.95</v>
       </c>
       <c r="Y23" t="n">
-        <v>1268.8</v>
+        <v>1547.9</v>
       </c>
       <c r="Z23" t="n">
-        <v>1205.45</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>951</v>
-      </c>
-      <c r="AB23" t="n">
-        <v>936.25</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>1044.85</v>
-      </c>
-      <c r="AD23" t="n">
-        <v>942.38</v>
-      </c>
-      <c r="AE23" t="n">
-        <v>947.75</v>
-      </c>
-      <c r="AF23" t="n">
-        <v>932.05</v>
-      </c>
-      <c r="AG23" t="n">
-        <v>949.4</v>
-      </c>
-      <c r="AH23" t="n">
-        <v>1003.4</v>
-      </c>
-      <c r="AI23" t="n">
-        <v>879.4</v>
+        <v>1483.45</v>
       </c>
     </row>
     <row r="24">
@@ -2830,47 +2235,22 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="W24" t="n">
-        <v>1283</v>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
       </c>
       <c r="X24" t="n">
-        <v>1156.08</v>
+        <v>703.63</v>
       </c>
       <c r="Y24" t="n">
-        <v>1210.3</v>
+        <v>751.2</v>
       </c>
       <c r="Z24" t="n">
-        <v>1159.2</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>726.73</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>899.05</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>989.88</v>
-      </c>
-      <c r="AD24" t="n">
-        <v>843.3</v>
-      </c>
-      <c r="AE24" t="n">
-        <v>750.15</v>
-      </c>
-      <c r="AF24" t="n">
-        <v>923.7</v>
-      </c>
-      <c r="AG24" t="n">
-        <v>861.95</v>
-      </c>
-      <c r="AH24" t="n">
-        <v>858.15</v>
-      </c>
-      <c r="AI24" t="n">
-        <v>1002.25</v>
+        <v>731.91</v>
       </c>
     </row>
     <row r="25">
@@ -2892,49 +2272,20 @@
       <c r="T25" t="n">
         <v>1558.9</v>
       </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="W25" t="n">
-        <v>1050.3</v>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
       </c>
       <c r="X25" t="n">
-        <v>1108.9</v>
+        <v>779.75</v>
       </c>
       <c r="Y25" t="n">
-        <v>1199</v>
+        <v>680.1</v>
       </c>
       <c r="Z25" t="n">
-        <v>1437.8</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>882.3</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>836.15</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>779.65</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>839.05</v>
-      </c>
-      <c r="AE25" t="n">
-        <v>914.25</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>938.4</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>800.05</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>826.25</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>1002.78</v>
+        <v>627.95</v>
       </c>
     </row>
     <row r="26">
@@ -2956,49 +2307,20 @@
       <c r="T26" t="n">
         <v>1664.35</v>
       </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="W26" t="n">
-        <v>828.48</v>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
       </c>
       <c r="X26" t="n">
-        <v>1167.8</v>
+        <v>951</v>
       </c>
       <c r="Y26" t="n">
-        <v>1131.5</v>
+        <v>1122.45</v>
       </c>
       <c r="Z26" t="n">
-        <v>1356.75</v>
-      </c>
-      <c r="AA26" t="n">
-        <v>708.53</v>
-      </c>
-      <c r="AB26" t="n">
-        <v>811.8</v>
-      </c>
-      <c r="AC26" t="n">
-        <v>768.35</v>
-      </c>
-      <c r="AD26" t="n">
-        <v>563.1</v>
-      </c>
-      <c r="AE26" t="n">
-        <v>645.1</v>
-      </c>
-      <c r="AF26" t="n">
-        <v>815.4</v>
-      </c>
-      <c r="AG26" t="n">
-        <v>735.15</v>
-      </c>
-      <c r="AH26" t="n">
-        <v>604.65</v>
-      </c>
-      <c r="AI26" t="n">
-        <v>776.4</v>
+        <v>566.05</v>
       </c>
     </row>
     <row r="27">
@@ -3020,49 +2342,20 @@
       <c r="T27" t="n">
         <v>1684.45</v>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="W27" t="n">
-        <v>885.45</v>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
       </c>
       <c r="X27" t="n">
-        <v>1227.11</v>
+        <v>726.73</v>
       </c>
       <c r="Y27" t="n">
-        <v>1329.9</v>
+        <v>1146.66</v>
       </c>
       <c r="Z27" t="n">
-        <v>1364.95</v>
-      </c>
-      <c r="AA27" t="n">
-        <v>735.95</v>
-      </c>
-      <c r="AB27" t="n">
-        <v>851.05</v>
-      </c>
-      <c r="AC27" t="n">
-        <v>858.65</v>
-      </c>
-      <c r="AD27" t="n">
-        <v>1004.25</v>
-      </c>
-      <c r="AE27" t="n">
-        <v>853.1</v>
-      </c>
-      <c r="AF27" t="n">
-        <v>849.95</v>
-      </c>
-      <c r="AG27" t="n">
-        <v>868.15</v>
-      </c>
-      <c r="AH27" t="n">
-        <v>951.3</v>
-      </c>
-      <c r="AI27" t="n">
-        <v>999.75</v>
+        <v>666.7</v>
       </c>
     </row>
     <row r="28">
@@ -3084,6 +2377,21 @@
       <c r="T28" t="n">
         <v>1686.1</v>
       </c>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X28" t="n">
+        <v>882.3</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>684.65</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>874.5</v>
+      </c>
     </row>
     <row r="29">
       <c r="M29" t="n">
@@ -3104,6 +2412,21 @@
       <c r="T29" t="n">
         <v>1111.15</v>
       </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X29" t="n">
+        <v>708.53</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>755.13</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>568.05</v>
+      </c>
     </row>
     <row r="30">
       <c r="M30" t="n">
@@ -3124,6 +2447,21 @@
       <c r="T30" t="n">
         <v>936.9</v>
       </c>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X30" t="n">
+        <v>735.95</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>837.9</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>744.95</v>
+      </c>
     </row>
     <row r="31">
       <c r="M31" t="n">
@@ -3144,6 +2482,25 @@
       <c r="T31" t="n">
         <v>1165.33</v>
       </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X31" t="n">
+        <v>811.75</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>665.3</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>898.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="M32" t="n">
@@ -3164,6 +2521,21 @@
       <c r="T32" t="n">
         <v>1475.4</v>
       </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
+        <v>564.95</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>541.65</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>555.55</v>
+      </c>
     </row>
     <row r="33">
       <c r="M33" t="n">
@@ -3184,6 +2556,21 @@
       <c r="T33" t="n">
         <v>1276.5</v>
       </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X33" t="n">
+        <v>936.25</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>559.5</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>771.45</v>
+      </c>
     </row>
     <row r="34">
       <c r="M34" t="n">
@@ -3204,6 +2591,21 @@
       <c r="T34" t="n">
         <v>1401.65</v>
       </c>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X34" t="n">
+        <v>899.05</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>469.65</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>768.48</v>
+      </c>
     </row>
     <row r="35">
       <c r="M35" t="n">
@@ -3224,6 +2626,21 @@
       <c r="T35" t="n">
         <v>1431.3</v>
       </c>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X35" t="n">
+        <v>836.15</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>662.7</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>736.9</v>
+      </c>
     </row>
     <row r="36">
       <c r="M36" t="n">
@@ -3244,6 +2661,21 @@
       <c r="T36" t="n">
         <v>1528.65</v>
       </c>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X36" t="n">
+        <v>811.8</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>583.05</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>671.3</v>
+      </c>
     </row>
     <row r="37">
       <c r="M37" t="n">
@@ -3264,6 +2696,21 @@
       <c r="T37" t="n">
         <v>1479</v>
       </c>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X37" t="n">
+        <v>851.05</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>556.75</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>730.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="M38" t="n">
@@ -3284,6 +2731,25 @@
       <c r="T38" t="n">
         <v>1168.55</v>
       </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X38" t="n">
+        <v>643.03</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>616.35</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>549.38</v>
+      </c>
     </row>
     <row r="39">
       <c r="M39" t="n">
@@ -3304,6 +2770,21 @@
       <c r="T39" t="n">
         <v>1869.15</v>
       </c>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X39" t="n">
+        <v>712.6</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>693.85</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>687.25</v>
+      </c>
     </row>
     <row r="40">
       <c r="M40" t="n">
@@ -3324,6 +2805,21 @@
       <c r="T40" t="n">
         <v>1822.66</v>
       </c>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X40" t="n">
+        <v>1044.85</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>611.1</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>752.75</v>
+      </c>
     </row>
     <row r="41">
       <c r="M41" t="n">
@@ -3344,6 +2840,21 @@
       <c r="T41" t="n">
         <v>1596.8</v>
       </c>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X41" t="n">
+        <v>989.88</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>615.5</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>535.23</v>
+      </c>
     </row>
     <row r="42">
       <c r="M42" t="n">
@@ -3364,6 +2875,21 @@
       <c r="T42" t="n">
         <v>1549.75</v>
       </c>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X42" t="n">
+        <v>779.65</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>524.55</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>530.85</v>
+      </c>
     </row>
     <row r="43">
       <c r="M43" t="n">
@@ -3384,6 +2910,21 @@
       <c r="T43" t="n">
         <v>1609.65</v>
       </c>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X43" t="n">
+        <v>768.35</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>567.4</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>737.25</v>
+      </c>
     </row>
     <row r="44">
       <c r="M44" t="n">
@@ -3404,6 +2945,21 @@
       <c r="T44" t="n">
         <v>1899.08</v>
       </c>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X44" t="n">
+        <v>858.65</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>616.15</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>737.75</v>
+      </c>
     </row>
     <row r="45">
       <c r="M45" t="n">
@@ -3424,6 +2980,25 @@
       <c r="T45" t="n">
         <v>1590.94</v>
       </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X45" t="n">
+        <v>849.9</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>734.3</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>845.33</v>
+      </c>
     </row>
     <row r="46">
       <c r="M46" t="n">
@@ -3444,6 +3019,21 @@
       <c r="T46" t="n">
         <v>1611.45</v>
       </c>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X46" t="n">
+        <v>609.65</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>607.2</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>661.05</v>
+      </c>
     </row>
     <row r="47">
       <c r="M47" t="n">
@@ -3464,6 +3054,21 @@
       <c r="T47" t="n">
         <v>1684.2</v>
       </c>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X47" t="n">
+        <v>942.38</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>710.9299999999999</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>640.03</v>
+      </c>
     </row>
     <row r="48">
       <c r="M48" t="n">
@@ -3484,6 +3089,21 @@
       <c r="T48" t="n">
         <v>1684.15</v>
       </c>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X48" t="n">
+        <v>843.3</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>659.25</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>677.25</v>
+      </c>
     </row>
     <row r="49">
       <c r="M49" t="n">
@@ -3504,6 +3124,21 @@
       <c r="T49" t="n">
         <v>1668.2</v>
       </c>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X49" t="n">
+        <v>839.05</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>631.8</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>841.8</v>
+      </c>
     </row>
     <row r="50">
       <c r="M50" t="n">
@@ -3524,6 +3159,21 @@
       <c r="T50" t="n">
         <v>1564.35</v>
       </c>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X50" t="n">
+        <v>563.1</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>639.85</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>725.1799999999999</v>
+      </c>
     </row>
     <row r="51">
       <c r="M51" t="n">
@@ -3544,6 +3194,21 @@
       <c r="T51" t="n">
         <v>1837.4</v>
       </c>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X51" t="n">
+        <v>1004.25</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>670.78</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>688.15</v>
+      </c>
     </row>
     <row r="52">
       <c r="M52" t="n">
@@ -3564,6 +3229,25 @@
       <c r="T52" t="n">
         <v>1716.95</v>
       </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X52" t="n">
+        <v>796.55</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>622.1</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>955.29</v>
+      </c>
     </row>
     <row r="53">
       <c r="M53" t="n">
@@ -3584,6 +3268,21 @@
       <c r="T53" t="n">
         <v>2257.06</v>
       </c>
+      <c r="V53" t="inlineStr"/>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X53" t="n">
+        <v>727.75</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>598.55</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>518.75</v>
+      </c>
     </row>
     <row r="54">
       <c r="M54" t="n">
@@ -3604,6 +3303,21 @@
       <c r="T54" t="n">
         <v>1753.88</v>
       </c>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X54" t="n">
+        <v>947.75</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>534.35</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="55">
       <c r="M55" t="n">
@@ -3624,6 +3338,21 @@
       <c r="T55" t="n">
         <v>1968.6</v>
       </c>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X55" t="n">
+        <v>750.15</v>
+      </c>
+      <c r="Y55" t="n">
+        <v>623.35</v>
+      </c>
+      <c r="Z55" t="n">
+        <v>734.78</v>
+      </c>
     </row>
     <row r="56">
       <c r="M56" t="n">
@@ -3644,6 +3373,21 @@
       <c r="T56" t="n">
         <v>2005.3</v>
       </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X56" t="n">
+        <v>914.25</v>
+      </c>
+      <c r="Y56" t="n">
+        <v>718.45</v>
+      </c>
+      <c r="Z56" t="n">
+        <v>865.05</v>
+      </c>
     </row>
     <row r="57">
       <c r="M57" t="n">
@@ -3664,6 +3408,21 @@
       <c r="T57" t="n">
         <v>1967</v>
       </c>
+      <c r="V57" t="inlineStr"/>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X57" t="n">
+        <v>645.1</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>433.9</v>
+      </c>
+      <c r="Z57" t="n">
+        <v>691.8</v>
+      </c>
     </row>
     <row r="58">
       <c r="M58" t="n">
@@ -3684,6 +3443,21 @@
       <c r="T58" t="n">
         <v>2242.85</v>
       </c>
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X58" t="n">
+        <v>853.1</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>508.4</v>
+      </c>
+      <c r="Z58" t="n">
+        <v>769.05</v>
+      </c>
     </row>
     <row r="59">
       <c r="M59" t="n">
@@ -3704,6 +3478,25 @@
       <c r="T59" t="n">
         <v>1461.05</v>
       </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X59" t="n">
+        <v>743.9</v>
+      </c>
+      <c r="Y59" t="n">
+        <v>675.9</v>
+      </c>
+      <c r="Z59" t="n">
+        <v>868.63</v>
+      </c>
     </row>
     <row r="60">
       <c r="M60" t="n">
@@ -3724,6 +3517,21 @@
       <c r="T60" t="n">
         <v>1197.25</v>
       </c>
+      <c r="V60" t="inlineStr"/>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X60" t="n">
+        <v>662.5</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>713.55</v>
+      </c>
+      <c r="Z60" t="n">
+        <v>576.15</v>
+      </c>
     </row>
     <row r="61">
       <c r="M61" t="n">
@@ -3744,6 +3552,21 @@
       <c r="T61" t="n">
         <v>1732.03</v>
       </c>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X61" t="n">
+        <v>932.05</v>
+      </c>
+      <c r="Y61" t="n">
+        <v>652.46</v>
+      </c>
+      <c r="Z61" t="n">
+        <v>728.65</v>
+      </c>
     </row>
     <row r="62">
       <c r="M62" t="n">
@@ -3764,6 +3587,21 @@
       <c r="T62" t="n">
         <v>1649.27</v>
       </c>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X62" t="n">
+        <v>923.7</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="Z62" t="n">
+        <v>708.05</v>
+      </c>
     </row>
     <row r="63">
       <c r="M63" t="n">
@@ -3784,6 +3622,21 @@
       <c r="T63" t="n">
         <v>1602.95</v>
       </c>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X63" t="n">
+        <v>938.4</v>
+      </c>
+      <c r="Y63" t="n">
+        <v>688.4</v>
+      </c>
+      <c r="Z63" t="n">
+        <v>776.5</v>
+      </c>
     </row>
     <row r="64">
       <c r="M64" t="n">
@@ -3804,6 +3657,21 @@
       <c r="T64" t="n">
         <v>1439.45</v>
       </c>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X64" t="n">
+        <v>815.4</v>
+      </c>
+      <c r="Y64" t="n">
+        <v>581.65</v>
+      </c>
+      <c r="Z64" t="n">
+        <v>620.65</v>
+      </c>
     </row>
     <row r="65">
       <c r="M65" t="n">
@@ -3824,6 +3692,21 @@
       <c r="T65" t="n">
         <v>1600.35</v>
       </c>
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X65" t="n">
+        <v>849.95</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>735.28</v>
+      </c>
+      <c r="Z65" t="n">
+        <v>622.1</v>
+      </c>
     </row>
     <row r="66">
       <c r="M66" t="n">
@@ -3844,6 +3727,25 @@
       <c r="T66" t="n">
         <v>1595.35</v>
       </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X66" t="n">
+        <v>827.55</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>655</v>
+      </c>
+      <c r="Z66" t="n">
+        <v>693.45</v>
+      </c>
     </row>
     <row r="67">
       <c r="M67" t="n">
@@ -3864,6 +3766,21 @@
       <c r="T67" t="n">
         <v>1537</v>
       </c>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X67" t="n">
+        <v>753.55</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>753.15</v>
+      </c>
+      <c r="Z67" t="n">
+        <v>398.85</v>
+      </c>
     </row>
     <row r="68">
       <c r="M68" t="n">
@@ -3884,6 +3801,21 @@
       <c r="T68" t="n">
         <v>1590.4</v>
       </c>
+      <c r="V68" t="inlineStr"/>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X68" t="n">
+        <v>949.4</v>
+      </c>
+      <c r="Y68" t="n">
+        <v>755.55</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>637.05</v>
+      </c>
     </row>
     <row r="69">
       <c r="M69" t="n">
@@ -3904,6 +3836,21 @@
       <c r="T69" t="n">
         <v>1282.05</v>
       </c>
+      <c r="V69" t="inlineStr"/>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X69" t="n">
+        <v>861.95</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>745.75</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>693.38</v>
+      </c>
     </row>
     <row r="70">
       <c r="M70" t="n">
@@ -3924,6 +3871,21 @@
       <c r="T70" t="n">
         <v>1954.8</v>
       </c>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X70" t="n">
+        <v>800.05</v>
+      </c>
+      <c r="Y70" t="n">
+        <v>629</v>
+      </c>
+      <c r="Z70" t="n">
+        <v>669.2</v>
+      </c>
     </row>
     <row r="71">
       <c r="M71" t="n">
@@ -3944,6 +3906,21 @@
       <c r="T71" t="n">
         <v>2159.08</v>
       </c>
+      <c r="V71" t="inlineStr"/>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X71" t="n">
+        <v>735.15</v>
+      </c>
+      <c r="Y71" t="n">
+        <v>573.95</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>448.45</v>
+      </c>
     </row>
     <row r="72">
       <c r="M72" t="n">
@@ -3964,6 +3941,21 @@
       <c r="T72" t="n">
         <v>1886.6</v>
       </c>
+      <c r="V72" t="inlineStr"/>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X72" t="n">
+        <v>868.15</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>839.05</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>578.45</v>
+      </c>
     </row>
     <row r="73">
       <c r="M73" t="n">
@@ -3984,6 +3976,25 @@
       <c r="T73" t="n">
         <v>1712.43</v>
       </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X73" t="n">
+        <v>714.55</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>516.45</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>374.04</v>
+      </c>
     </row>
     <row r="74">
       <c r="M74" t="n">
@@ -4004,6 +4015,21 @@
       <c r="T74" t="n">
         <v>1977.5</v>
       </c>
+      <c r="V74" t="inlineStr"/>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X74" t="n">
+        <v>735.9</v>
+      </c>
+      <c r="Y74" t="n">
+        <v>562.25</v>
+      </c>
+      <c r="Z74" t="n">
+        <v>210.95</v>
+      </c>
     </row>
     <row r="75">
       <c r="M75" t="n">
@@ -4024,6 +4050,21 @@
       <c r="T75" t="n">
         <v>2215.11</v>
       </c>
+      <c r="V75" t="inlineStr"/>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X75" t="n">
+        <v>1003.4</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>708.35</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>383.85</v>
+      </c>
     </row>
     <row r="76">
       <c r="M76" t="n">
@@ -4044,6 +4085,21 @@
       <c r="T76" t="n">
         <v>1751.36</v>
       </c>
+      <c r="V76" t="inlineStr"/>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X76" t="n">
+        <v>858.15</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>648.38</v>
+      </c>
+      <c r="Z76" t="n">
+        <v>413.75</v>
+      </c>
     </row>
     <row r="77">
       <c r="M77" t="n">
@@ -4064,6 +4120,21 @@
       <c r="T77" t="n">
         <v>1644.85</v>
       </c>
+      <c r="V77" t="inlineStr"/>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X77" t="n">
+        <v>826.25</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>750.45</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>273.7</v>
+      </c>
     </row>
     <row r="78">
       <c r="M78" t="n">
@@ -4084,6 +4155,21 @@
       <c r="T78" t="n">
         <v>1805.68</v>
       </c>
+      <c r="V78" t="inlineStr"/>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X78" t="n">
+        <v>604.65</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>570.3</v>
+      </c>
+      <c r="Z78" t="n">
+        <v>282.8</v>
+      </c>
     </row>
     <row r="79">
       <c r="M79" t="n">
@@ -4104,6 +4190,21 @@
       <c r="T79" t="n">
         <v>1724.85</v>
       </c>
+      <c r="V79" t="inlineStr"/>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X79" t="n">
+        <v>951.3</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>657.1799999999999</v>
+      </c>
+      <c r="Z79" t="n">
+        <v>390.95</v>
+      </c>
     </row>
     <row r="80">
       <c r="M80" t="n">
@@ -4124,6 +4225,25 @@
       <c r="T80" t="n">
         <v>1805.28</v>
       </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X80" t="n">
+        <v>733.3099999999999</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>524.2</v>
+      </c>
+      <c r="Z80" t="n">
+        <v>60.51</v>
+      </c>
     </row>
     <row r="81">
       <c r="M81" t="n">
@@ -4144,6 +4264,21 @@
       <c r="T81" t="n">
         <v>1733.4</v>
       </c>
+      <c r="V81" t="inlineStr"/>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X81" t="n">
+        <v>811.7</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>552</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="M82" t="n">
@@ -4164,6 +4299,21 @@
       <c r="T82" t="n">
         <v>1929.63</v>
       </c>
+      <c r="V82" t="inlineStr"/>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X82" t="n">
+        <v>879.4</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>605.35</v>
+      </c>
+      <c r="Z82" t="n">
+        <v>84.95</v>
+      </c>
     </row>
     <row r="83">
       <c r="M83" t="n">
@@ -4184,6 +4334,21 @@
       <c r="T83" t="n">
         <v>1890.3</v>
       </c>
+      <c r="V83" t="inlineStr"/>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X83" t="n">
+        <v>1002.25</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>520.1</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>116.02</v>
+      </c>
     </row>
     <row r="84">
       <c r="M84" t="n">
@@ -4204,6 +4369,21 @@
       <c r="T84" t="n">
         <v>2145.95</v>
       </c>
+      <c r="V84" t="inlineStr"/>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X84" t="n">
+        <v>1002.78</v>
+      </c>
+      <c r="Y84" t="n">
+        <v>506.15</v>
+      </c>
+      <c r="Z84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="M85" t="n">
@@ -4224,6 +4404,21 @@
       <c r="T85" t="n">
         <v>1933.38</v>
       </c>
+      <c r="V85" t="inlineStr"/>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X85" t="n">
+        <v>776.4</v>
+      </c>
+      <c r="Y85" t="n">
+        <v>550.78</v>
+      </c>
+      <c r="Z85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="M86" t="n">
@@ -4244,6 +4439,21 @@
       <c r="T86" t="n">
         <v>2097.75</v>
       </c>
+      <c r="V86" t="inlineStr"/>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X86" t="n">
+        <v>999.75</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>613.7</v>
+      </c>
+      <c r="Z86" t="n">
+        <v>31.05</v>
+      </c>
     </row>
     <row r="87">
       <c r="M87" t="n">
@@ -4264,6 +4474,25 @@
       <c r="T87" t="n">
         <v>2244.95</v>
       </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="X87" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>287.1</v>
+      </c>
+      <c r="Z87" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="88">
       <c r="M88" t="n">
@@ -4284,6 +4513,21 @@
       <c r="T88" t="n">
         <v>2154.7</v>
       </c>
+      <c r="V88" t="inlineStr"/>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>339.5</v>
+      </c>
+      <c r="Z88" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="89">
       <c r="M89" t="n">
@@ -4304,6 +4548,21 @@
       <c r="T89" t="n">
         <v>2437.4</v>
       </c>
+      <c r="V89" t="inlineStr"/>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="X89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z89" t="n">
+        <v>46.5</v>
+      </c>
     </row>
     <row r="90">
       <c r="M90" t="n">
@@ -4324,6 +4583,21 @@
       <c r="T90" t="n">
         <v>1524.95</v>
       </c>
+      <c r="V90" t="inlineStr"/>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y90" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="Z90" t="n">
+        <v>33.77</v>
+      </c>
     </row>
     <row r="91">
       <c r="M91" t="n">
@@ -4344,6 +4618,21 @@
       <c r="T91" t="n">
         <v>1299.45</v>
       </c>
+      <c r="V91" t="inlineStr"/>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="X91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>111.1</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="M92" t="n">
@@ -4363,6 +4652,38 @@
       </c>
       <c r="T92" t="n">
         <v>1768.74</v>
+      </c>
+      <c r="V92" t="inlineStr"/>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y92" t="n">
+        <v>135.88</v>
+      </c>
+      <c r="Z92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="V93" t="inlineStr"/>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z93" t="n">
+        <v>39.4</v>
       </c>
     </row>
   </sheetData>
@@ -4410,88 +4731,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="60" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Key Observations</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Automated findings highlighting significant trends and patterns with identified areas for action.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:E3"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="60" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Key Observations</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Automated findings highlighting significant trends and patterns with identified areas for action.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:E3"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>